<commit_message>
updated mtech alumini data
</commit_message>
<xml_diff>
--- a/excels/Phd_Alumini.xlsx
+++ b/excels/Phd_Alumini.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Documents\PA_catts(A)\mainnn\NITW-Transportation-Division-main\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw deploy\NITW-Transportation-Division-main\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE4FAE7A-E3E2-417F-92D8-560673911373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" firstSheet="5" activeTab="22"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1980" sheetId="1" r:id="rId1"/>
@@ -249,9 +250,6 @@
     <t>Prof. C.S.R.K. Prasad</t>
   </si>
   <si>
-    <t>https://nitw.irins.org/profile_images/156343.JPG</t>
-  </si>
-  <si>
     <t>D. Abhigna</t>
   </si>
   <si>
@@ -1402,11 +1400,14 @@
   <si>
     <t>Retd. Chief Engineer (Roads Wing), Chief Executive of L.R. Kadiyali &amp; Associates (New Delhi)</t>
   </si>
+  <si>
+    <t>https://erp.nitw.ac.in/ext/profile/getUserImage/ce-ss</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="19">
     <font>
       <sz val="11"/>
@@ -1879,7 +1880,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1901,10 +1902,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -1913,7 +1914,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -1927,10 +1928,10 @@
         <v>7</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>8</v>
@@ -1942,7 +1943,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1962,10 +1963,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -1974,7 +1975,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -1988,19 +1989,19 @@
         <v>29</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>266</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>267</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75">
@@ -2012,7 +2013,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2033,10 +2034,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2045,7 +2046,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="60">
@@ -2059,14 +2060,14 @@
         <v>31</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5">
@@ -2080,31 +2081,31 @@
         <v>33</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>264</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>265</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G3" r:id="rId1"/>
+    <hyperlink ref="G3" r:id="rId1" xr:uid="{00000000-0004-0000-0A00-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2123,10 +2124,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2135,7 +2136,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -2149,19 +2150,19 @@
         <v>35</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>36</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="H2" s="24" t="s">
         <v>318</v>
-      </c>
-      <c r="H2" s="24" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5">
@@ -2175,19 +2176,19 @@
         <v>38</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G3" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>324</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5">
@@ -2201,19 +2202,19 @@
         <v>41</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>36</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2226,7 +2227,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2244,10 +2245,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2256,7 +2257,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -2270,10 +2271,10 @@
         <v>43</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>39</v>
@@ -2285,7 +2286,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -2300,10 +2301,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2312,7 +2313,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -2326,19 +2327,19 @@
         <v>45</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>320</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>321</v>
       </c>
     </row>
   </sheetData>
@@ -2347,7 +2348,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2365,10 +2366,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2377,7 +2378,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -2391,17 +2392,17 @@
         <v>47</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>39</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5">
@@ -2415,10 +2416,10 @@
         <v>49</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>39</v>
@@ -2431,7 +2432,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2450,10 +2451,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2462,7 +2463,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="315">
@@ -2476,14 +2477,14 @@
         <v>51</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
         <v>36</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5">
@@ -2497,10 +2498,10 @@
         <v>53</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>36</v>
@@ -2513,7 +2514,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2531,10 +2532,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2543,7 +2544,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -2557,10 +2558,10 @@
         <v>55</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>36</v>
@@ -2578,10 +2579,10 @@
         <v>57</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>236</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>237</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>36</v>
@@ -2594,7 +2595,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2615,10 +2616,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2627,7 +2628,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -2641,10 +2642,10 @@
         <v>59</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>36</v>
@@ -2660,7 +2661,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2681,10 +2682,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2693,7 +2694,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -2707,10 +2708,10 @@
         <v>61</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>36</v>
@@ -2723,7 +2724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2741,10 +2742,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2753,7 +2754,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -2767,19 +2768,19 @@
         <v>10</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>227</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -2788,7 +2789,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2807,10 +2808,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2819,7 +2820,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -2833,28 +2834,31 @@
         <v>63</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="G2" t="s">
-        <v>65</v>
+      <c r="G2" s="4" t="s">
+        <v>333</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{7E855022-3677-4B98-BC3F-56FC82084663}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2874,10 +2878,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2886,7 +2890,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -2894,22 +2898,22 @@
         <v>2018</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>68</v>
-      </c>
       <c r="G2" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -2918,7 +2922,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2938,10 +2942,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -2950,7 +2954,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -2958,22 +2962,22 @@
         <v>2019</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>71</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5">
@@ -2981,22 +2985,22 @@
         <v>2019</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>73</v>
-      </c>
       <c r="D3" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>64</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5">
@@ -3004,22 +3008,22 @@
         <v>2019</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>75</v>
-      </c>
       <c r="D4" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>64</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="409.5">
@@ -3027,22 +3031,22 @@
         <v>2019</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="D5" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>64</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="409.5">
@@ -3050,22 +3054,22 @@
         <v>2019</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>79</v>
-      </c>
       <c r="D6" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="409.5">
@@ -3073,22 +3077,22 @@
         <v>2019</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>82</v>
-      </c>
       <c r="G7" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>
@@ -3097,7 +3101,7 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3121,10 +3125,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="14" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="14" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>3</v>
@@ -3133,7 +3137,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -3141,22 +3145,22 @@
         <v>2020</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="12" t="s">
-        <v>84</v>
-      </c>
       <c r="D2" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5">
@@ -3164,22 +3168,22 @@
         <v>2020</v>
       </c>
       <c r="B3" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="D3" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="F3" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D3" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>252</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>87</v>
-      </c>
       <c r="G3" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5">
@@ -3187,22 +3191,22 @@
         <v>2020</v>
       </c>
       <c r="B4" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="C4" s="12" t="s">
-        <v>89</v>
-      </c>
       <c r="D4" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
   </sheetData>
@@ -3211,7 +3215,7 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3230,10 +3234,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>3</v>
@@ -3242,7 +3246,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -3250,22 +3254,22 @@
         <v>2021</v>
       </c>
       <c r="B2" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>91</v>
-      </c>
       <c r="D2" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="H2" s="7"/>
     </row>
@@ -3274,22 +3278,22 @@
         <v>2021</v>
       </c>
       <c r="B3" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>93</v>
-      </c>
       <c r="D3" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>64</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H3" s="7"/>
     </row>
@@ -3298,22 +3302,22 @@
         <v>2021</v>
       </c>
       <c r="B4" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>95</v>
-      </c>
       <c r="D4" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H4" s="7"/>
     </row>
@@ -3323,7 +3327,7 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3344,10 +3348,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3356,7 +3360,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.5">
@@ -3364,22 +3368,22 @@
         <v>2022</v>
       </c>
       <c r="B2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5">
@@ -3387,22 +3391,22 @@
         <v>2022</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5">
@@ -3410,22 +3414,22 @@
         <v>2022</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>98</v>
-      </c>
       <c r="D4" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="409.5">
@@ -3433,22 +3437,22 @@
         <v>2022</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>100</v>
-      </c>
       <c r="D5" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>64</v>
       </c>
       <c r="G5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="409.5">
@@ -3456,22 +3460,22 @@
         <v>2022</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>102</v>
-      </c>
       <c r="D6" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>64</v>
       </c>
       <c r="G6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="409.5">
@@ -3479,22 +3483,22 @@
         <v>2022</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>104</v>
-      </c>
       <c r="D7" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="409.5">
@@ -3502,22 +3506,22 @@
         <v>2022</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -3526,7 +3530,7 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3547,10 +3551,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3559,7 +3563,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -3567,19 +3571,19 @@
         <v>2023</v>
       </c>
       <c r="B2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5">
@@ -3587,22 +3591,22 @@
         <v>2023</v>
       </c>
       <c r="B3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5">
@@ -3610,16 +3614,16 @@
         <v>2023</v>
       </c>
       <c r="B4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -3628,7 +3632,7 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3649,10 +3653,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3661,7 +3665,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -3669,22 +3673,22 @@
         <v>2024</v>
       </c>
       <c r="B2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F2" t="s">
+        <v>186</v>
+      </c>
+      <c r="G2" t="s">
         <v>187</v>
-      </c>
-      <c r="G2" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5">
@@ -3692,19 +3696,19 @@
         <v>2024</v>
       </c>
       <c r="B3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5">
@@ -3712,22 +3716,22 @@
         <v>2024</v>
       </c>
       <c r="B4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="F4" t="s">
         <v>192</v>
       </c>
-      <c r="D4" t="s">
-        <v>119</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>285</v>
-      </c>
-      <c r="F4" t="s">
-        <v>193</v>
-      </c>
       <c r="G4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="409.5">
@@ -3735,19 +3739,19 @@
         <v>2024</v>
       </c>
       <c r="B5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="409.5">
@@ -3755,22 +3759,22 @@
         <v>2024</v>
       </c>
       <c r="B6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C6" t="s">
+        <v>312</v>
+      </c>
+      <c r="D6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="F6" t="s">
+        <v>186</v>
+      </c>
+      <c r="G6" t="s">
         <v>313</v>
-      </c>
-      <c r="D6" t="s">
-        <v>121</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>254</v>
-      </c>
-      <c r="F6" t="s">
-        <v>187</v>
-      </c>
-      <c r="G6" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75">
@@ -3778,19 +3782,19 @@
         <v>2024</v>
       </c>
       <c r="B7" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G7" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="409.5">
@@ -3798,22 +3802,22 @@
         <v>2024</v>
       </c>
       <c r="B8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C8" t="s">
+        <v>195</v>
+      </c>
+      <c r="D8" t="s">
+        <v>122</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>277</v>
+      </c>
+      <c r="F8" t="s">
+        <v>184</v>
+      </c>
+      <c r="G8" t="s">
         <v>196</v>
-      </c>
-      <c r="D8" t="s">
-        <v>123</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>278</v>
-      </c>
-      <c r="F8" t="s">
-        <v>185</v>
-      </c>
-      <c r="G8" t="s">
-        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -3822,7 +3826,7 @@
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3845,10 +3849,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -3857,7 +3861,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -3865,19 +3869,19 @@
         <v>2025</v>
       </c>
       <c r="B2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="409.5">
@@ -3885,22 +3889,22 @@
         <v>2025</v>
       </c>
       <c r="B3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C3" t="s">
+        <v>180</v>
+      </c>
+      <c r="D3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="F3" t="s">
+        <v>182</v>
+      </c>
+      <c r="G3" t="s">
         <v>181</v>
-      </c>
-      <c r="D3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>282</v>
-      </c>
-      <c r="F3" t="s">
-        <v>183</v>
-      </c>
-      <c r="G3" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="409.5">
@@ -3908,22 +3912,22 @@
         <v>2025</v>
       </c>
       <c r="B4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F4" t="s">
+        <v>182</v>
+      </c>
+      <c r="G4" t="s">
         <v>183</v>
-      </c>
-      <c r="G4" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="409.5">
@@ -3931,22 +3935,22 @@
         <v>2025</v>
       </c>
       <c r="B5" t="s">
+        <v>221</v>
+      </c>
+      <c r="C5" t="s">
         <v>222</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>222</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>223</v>
-      </c>
-      <c r="D5" t="s">
-        <v>223</v>
-      </c>
-      <c r="E5" s="19" t="s">
-        <v>290</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>273</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="409.5">
@@ -3954,31 +3958,31 @@
         <v>2025</v>
       </c>
       <c r="B6" t="s">
+        <v>285</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>287</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>286</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="F6" s="17" t="s">
         <v>288</v>
       </c>
-      <c r="E6" s="10" t="s">
-        <v>287</v>
-      </c>
-      <c r="F6" s="17" t="s">
-        <v>289</v>
-      </c>
       <c r="G6" s="20" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G5" r:id="rId1"/>
+    <hyperlink ref="G5" r:id="rId1" xr:uid="{00000000-0004-0000-1B00-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -3998,10 +4002,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4010,7 +4014,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -4018,34 +4022,34 @@
         <v>2026</v>
       </c>
       <c r="B2" s="21" t="s">
+        <v>306</v>
+      </c>
+      <c r="C2" s="22" t="s">
         <v>307</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="D2" s="22" t="s">
+        <v>311</v>
+      </c>
+      <c r="E2" s="10" t="s">
         <v>308</v>
       </c>
-      <c r="D2" s="22" t="s">
-        <v>312</v>
-      </c>
-      <c r="E2" s="10" t="s">
+      <c r="F2" s="22" t="s">
         <v>309</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="G2" s="23" t="s">
         <v>310</v>
-      </c>
-      <c r="G2" s="23" t="s">
-        <v>311</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1"/>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{00000000-0004-0000-1C00-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -4063,10 +4067,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4075,7 +4079,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -4089,19 +4093,19 @@
         <v>13</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>330</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -4110,7 +4114,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -4129,10 +4133,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4141,7 +4145,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -4155,16 +4159,16 @@
         <v>15</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
   </sheetData>
@@ -4173,7 +4177,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -4188,10 +4192,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4200,7 +4204,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -4214,19 +4218,19 @@
         <v>17</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>332</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>333</v>
       </c>
     </row>
   </sheetData>
@@ -4235,7 +4239,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -4253,10 +4257,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4265,7 +4269,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -4279,10 +4283,10 @@
         <v>19</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -4294,7 +4298,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -4309,10 +4313,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4321,7 +4325,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -4335,10 +4339,10 @@
         <v>21</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -4350,7 +4354,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -4372,10 +4376,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4384,7 +4388,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="90">
@@ -4398,7 +4402,7 @@
         <v>23</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
@@ -4410,19 +4414,19 @@
         <v>1989</v>
       </c>
       <c r="B3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="L3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -4431,7 +4435,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -4452,10 +4456,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>215</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4464,7 +4468,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.5">
@@ -4478,10 +4482,10 @@
         <v>25</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -4498,17 +4502,17 @@
         <v>27</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="G3" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>327</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>328</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated phd alumini data
</commit_message>
<xml_diff>
--- a/excels/Phd_Alumini.xlsx
+++ b/excels/Phd_Alumini.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw deploy\NITW-Transportation-Division-main\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE4FAE7A-E3E2-417F-92D8-560673911373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A4D413-4571-4E57-89B3-57201BDEE956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1980" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="336">
   <si>
     <t>Year</t>
   </si>
@@ -1399,6 +1399,12 @@
   </si>
   <si>
     <t>Retd. Chief Engineer (Roads Wing), Chief Executive of L.R. Kadiyali &amp; Associates (New Delhi)</t>
+  </si>
+  <si>
+    <t>This study develops a scientific methodology for assessing rural and regional travel demand, determining optimal depot fleet sizes, and identifying strategic depot locations for public road transport corporations like APSRTC. The approach combines information minimization techniques using Conductors Statistical Records (CSR) for inter-zonal travel with socio-economic trip-rate modeling for intra-zonal travel. By analyzing 94 bus depots in Andhra Pradesh, the study identifies a non-linear relationship between fleet size and operational costs, establishing an optimal fleet size range that minimizes total investment and operational costs. Strategic depot locations are selected using Centrality Place Theory and a linear programming transportation model to minimize total travel costs within defined reach distances. Validation in the 9-district Hyderabad region demonstrates high model accuracy, offering a structured, data-driven framework for public transport corporations to optimize resource allocation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phd_Alumini/S2023/Lalam Govinda </t>
   </si>
   <si>
     <t>https://erp.nitw.ac.in/ext/profile/getUserImage/ce-ss</t>
@@ -2843,7 +2849,7 @@
         <v>64</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>274</v>
@@ -2851,7 +2857,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{7E855022-3677-4B98-BC3F-56FC82084663}"/>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{A5E065B3-B151-446B-AFAE-9D4FBBD0510F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3625,6 +3631,9 @@
       <c r="F4" t="s">
         <v>197</v>
       </c>
+      <c r="G4" t="s">
+        <v>334</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4491,7 +4500,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="90">
+    <row r="3" spans="1:8" ht="240">
       <c r="A3" s="3">
         <v>1992</v>
       </c>
@@ -4504,7 +4513,9 @@
       <c r="D3" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="E3" s="3"/>
+      <c r="E3" s="3" t="s">
+        <v>333</v>
+      </c>
       <c r="F3" s="3" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
phd alumini data update
</commit_message>
<xml_diff>
--- a/excels/Phd_Alumini.xlsx
+++ b/excels/Phd_Alumini.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw deploy\NITW-Transportation-Division-main\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NIT\Documents\PA_Catts\Nitw_WB\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A4D413-4571-4E57-89B3-57201BDEE956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A356362C-E90A-4F6A-B1F5-C0442C662899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1980" sheetId="1" r:id="rId1"/>
@@ -48,12 +48,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="337">
   <si>
     <t>Year</t>
   </si>
@@ -1401,20 +1404,43 @@
     <t>Retd. Chief Engineer (Roads Wing), Chief Executive of L.R. Kadiyali &amp; Associates (New Delhi)</t>
   </si>
   <si>
-    <t>This study develops a scientific methodology for assessing rural and regional travel demand, determining optimal depot fleet sizes, and identifying strategic depot locations for public road transport corporations like APSRTC. The approach combines information minimization techniques using Conductors Statistical Records (CSR) for inter-zonal travel with socio-economic trip-rate modeling for intra-zonal travel. By analyzing 94 bus depots in Andhra Pradesh, the study identifies a non-linear relationship between fleet size and operational costs, establishing an optimal fleet size range that minimizes total investment and operational costs. Strategic depot locations are selected using Centrality Place Theory and a linear programming transportation model to minimize total travel costs within defined reach distances. Validation in the 9-district Hyderabad region demonstrates high model accuracy, offering a structured, data-driven framework for public transport corporations to optimize resource allocation.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Phd_Alumini/S2023/Lalam Govinda </t>
   </si>
   <si>
     <t>https://erp.nitw.ac.in/ext/profile/getUserImage/ce-ss</t>
+  </si>
+  <si>
+    <t>As the urban travel demand continues to increase it is inconceivable that improvements in the existing transportation system alone could provide adequate transportation facilities for all the commuters. Magnitude of increases in transportation usage together with the deficiencies in the existing bus transportation system indicate that considerable additional capacity is required to be provided in various other forms. Laying of high capacity mass transit system such as Electric Multiple Unit need heavy investments disproportionate to the demand and they cannot be accommodated on city streets. Thus the most pressing problem facing the metropolitan cities is to introduce a medium capacity moderate investment oriented system that could be layed along the established high dense corridors of the metropolitan cities. The newly emerging Light Rail Transit technology appears to be a reasonably good solution which is not only capable of commuting 10000-20000 persons during peak hour per direction, but also can work and coexist together with the already existing Bus Route system. One of the main issues that confront in the introduction of LRT is the lack of a systematic approach in designing bus transit networks together with LRT network. A comprehensive and continuous appraisal throughout the evaluation, planning, design, implementation and management of LRT and the bus system is very much impending. The existing approaches fail to provide a handy tool in this direction.
+The purpose of this research is to propose an Integrated Approach on a macro level basis, with planners intervention. The main task is to integrate all types of mass transportation systems at the planning stage itself and to test a variety of alternatives with suggested performance indicators to eliminate wasteful duplication. The proposed frame work comprises of three main sub models.
+The Mass Transport Demand Estimation Model is proposed for finding the potential transit users on a variety mass transit options. Multinomial Logit Model is to be used in a simplified procedure to arrive at the mode split of all the competing modes. The future mass transit desire is to be computed from the total O-D Matrix obtained from landuse transport model with the help of the Logit model. The mass transit desire forms the basis for the route generation process.
+A transit network can be developed by The Alternate Route Generation Model by using total Origin-Destination Matrix. Alignment of new routes, integrating them with existing routes and evaluating the resulting network are the three important stages at this level. Results of the evaluation are then compared with the set of objectives and the policy in respect of additional routes or frequency or both is changed until satisfactory results are achieved for the final selection of the transit network. The Transit Route Generation Algorithm identifies LRT routes along with bus transit network and estimates the transit patronage for the combined network system.
+The Scheduling Model selects the optimal headways taking into consideration the marginal ridership concept which utilises the optimal fleet size to derive full benefits and consumer satisfaction.
+All the models fit into the overall urban transportation planning process and thus presents a simplified working tool in association with standard network coding procedures. Relevant computer programs are presented in FORTRAN language to make the methodology operational both on main frame as well as Personal Computers. These models include MASDEM for mass transit demand estimation, TRAB for transit building network, TRAN for transit analysis programme. The other models MICAS, TEMPLATE and MARIS are used for transit corridor identification and for suggesting mass transport management measures.
+The main feature of the study is that, it envisages an overall planning and management of mass transport systems through a systematic procedure ensuring healthy interaction between LRT and Bus system. All these models are subjected to a set of tests with the actual data obtained from the city of Hyderabad. The typical transport problems present in the city has provided an ideal setting for the case study. The complete package is applied to Hyderabad city to examine the operational difficulties and it is observed that the proposed approach is workable and will be of great help to planners in improving the efficiency of transit planning.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The present research work is concerned with the most appropriate and desirable sizing and location of "Bus Depots" or "Garages" and their spatial dispersion in a given region to meet the travel requirements of the people while providing the highest operational efficiency to the Transport Organisations. 
+Location of Bus Depots has acquired such a profound importance that not only the transport organisations are seized of the issue but also the people who harbour an inherent belief that the location of a bus depot in their area relieves them of their travel inconveniences. This belief to a great extent is well founded in the sense that the depots really have an important role to play in virtually translating their travel aspirations into reality through managerial policies. 
+In the course of this study it is noticed that adequately defined procedures are not evidenced in transport organisations for depot locations in relation to the available patterns of travel demand. 
+Fleet size is found to be varying widely from one depot to another while the depot managers and divisional managers prefer a depot size that supports a maximum staff strength of 500 to 600. Standardisation of fleet strength for a bus depot appears to be an urgent need to satisfactorily correlate the operational efficiency and the travel demand. 
+While the passengers do travel with varied trip lengths, it is found during the course of the study that the travel pattern at regional level can be broadly classified into two distinct categories: one the long distance and the other very short distance. Therefore, it is imperative that the bus operations need to be designed to satisfy both these requirements. It is observed during the study that the depot managers have a tendency to favour long distance services at the expense of short distance services for the obvious reason that the performance of the former is superior to the latter. The study further revealed that it is equally important to satisfy the needs of the short distance local travel and hence a trade off between the travel desires and operational performances is to be considered in all respects to arrive at an appropriate fleet mix. The study also revealed that the transport organisations have not yet focused their attention on the need to assess the total travel requirements, which alone can determine the reliable fleet estimates and assigning vehicles to various depots. 
+The size, number and dispersal of the depots in a region has significant impact on the total cost of operations for the organisation. There could be an optimal cost surface of these parameters which will yield best productivity results for the system. 
+The research presented provides an hypothesis for estimating the travel demand, determining the size and number of depots and their location in a region for their best operational efficiency. The proposed approach is formulated in 3 modules. 
+Module-I presents the quantification procedures of the short and long distance bus travel. The long distance travel between the identified traffic zones is proposed by Internal Volume Forecasting Models employing link Bus Volume data obtained through Conductors Statistical Returns. The demand for short distance travel within a zone is proposed by developing a relationship between the socio-economic and demographic indicators and the per capita trip rate of the people of the delineated sub-zones. 
+Module-II presents the procedure to assess the required number of buses to meet the long and short distance travel as established in Module I. The procedure takes into account several operational parameters such as speeds, turn around time, crew reporting and rest times and so on. It also includes overage seating capacity, vehicle utilisation, occupation ratio that are in vogue in the region. A procedure for desirable proportioning of the short and long haul buses is proposed by superimposing the performance of inter and intra zonal services on a common graph. Further, a viable size of a depot can be established through a study of cost, revenue and productivity parameters.
+Module-III provides a procedure to identify the candidate locations for depots based on the hierarchical trip generations and by determining ideal combination of locations minimising the total cost of operations, through an optimisation program. A procedure is also presented giving the best combination of fleet and number of depots in the Region. 
+The proposed hypothesis and the techniques are then applied to the Hyderabad region consisting of 10 districts which is presently covered by bus operations from Golconda and Kakatiya regions of APSRTC. Several studies are organised in this region to ascertain the present practices, the bus link volumes through CSR's, trip length frequencies, village level Home Interview Surveys, and opinion poll surveys of Depot and Divisional Managers. In addition, the information from secondary sources and depot records are gathered from as many as 44 depots in this area. The travel demand models are validated from a set of data not employed in the calibration and the results are found to be within acceptable limits of accuracy. 
+Based on the suggested procedure, the total fleet, fleet mix, viable depot size, number of depots and their locations are all computed for the base year as well as for the horizon years 1993 and 2001 respectively. 
+It is revealed that there could be a better location of the depots, than what is being practiced now, to give a greater level of service and at much lower investment costs. Even the priorities incorporated and implemented practiced for establishing the depots in the past few years need to be re-examined in the light of the results obtained in this study. 
+There is ample scope to further improve the model presented in this research by encompassing the issues concerned with Zoning, Calibration of local and long distance travel along with a number of measurement problems associated with them. 
+As there are gaps between the model attempting to explain the travel behaviour and those observed in reality, sincere efforts are required to study the micro level interfacing based on accurate documentation procedures at depot level on cost of operation. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1888,7 +1914,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.5703125" customWidth="1"/>
     <col min="3" max="5" width="42.28515625" customWidth="1"/>
@@ -1897,7 +1923,7 @@
     <col min="8" max="8" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1923,7 +1949,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1980</v>
       </c>
@@ -1951,14 +1977,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="21.42578125" customWidth="1"/>
     <col min="5" max="5" width="48" customWidth="1"/>
     <col min="7" max="7" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1984,7 +2010,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1996</v>
       </c>
@@ -2010,7 +2036,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75">
+    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="G3" s="2"/>
     </row>
   </sheetData>
@@ -2021,7 +2047,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="21.85546875" customWidth="1"/>
     <col min="5" max="5" width="44.140625" customWidth="1"/>
@@ -2029,7 +2055,7 @@
     <col min="7" max="7" width="20.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2055,7 +2081,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="60">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1997</v>
       </c>
@@ -2068,7 +2094,9 @@
       <c r="D2" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="E2" s="3"/>
+      <c r="E2" s="3" t="s">
+        <v>335</v>
+      </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
@@ -2076,7 +2104,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1997</v>
       </c>
@@ -2113,13 +2141,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27.42578125" customWidth="1"/>
     <col min="5" max="5" width="157.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2145,7 +2173,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1998</v>
       </c>
@@ -2171,7 +2199,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1998</v>
       </c>
@@ -2197,7 +2225,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1998</v>
       </c>
@@ -2223,7 +2251,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
     </row>
@@ -2235,12 +2263,12 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="23.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2266,7 +2294,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1999</v>
       </c>
@@ -2294,9 +2322,9 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2322,7 +2350,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2000</v>
       </c>
@@ -2356,12 +2384,12 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="38.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2387,7 +2415,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2001</v>
       </c>
@@ -2411,7 +2439,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2001</v>
       </c>
@@ -2440,13 +2468,13 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="60.28515625" customWidth="1"/>
     <col min="6" max="6" width="37" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2472,7 +2500,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="315">
+    <row r="2" spans="1:8" ht="315" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2003</v>
       </c>
@@ -2493,7 +2521,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2003</v>
       </c>
@@ -2522,12 +2550,12 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2553,7 +2581,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2004</v>
       </c>
@@ -2574,7 +2602,7 @@
       </c>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2004</v>
       </c>
@@ -2603,7 +2631,7 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="24.7109375" customWidth="1"/>
     <col min="4" max="4" width="23.42578125" customWidth="1"/>
@@ -2611,7 +2639,7 @@
     <col min="6" max="6" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2637,7 +2665,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2005</v>
       </c>
@@ -2658,7 +2686,7 @@
       </c>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:8" ht="15.75">
+    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="G3" s="2"/>
     </row>
   </sheetData>
@@ -2669,7 +2697,7 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.5703125" customWidth="1"/>
     <col min="3" max="3" width="27.7109375" customWidth="1"/>
@@ -2677,7 +2705,7 @@
     <col min="5" max="5" width="48.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2703,7 +2731,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2006</v>
       </c>
@@ -2732,12 +2760,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="5" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2763,7 +2791,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1982</v>
       </c>
@@ -2797,13 +2825,13 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="45.5703125" customWidth="1"/>
     <col min="8" max="8" width="40.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2829,7 +2857,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2012</v>
       </c>
@@ -2848,17 +2876,14 @@
       <c r="F2" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>335</v>
+      <c r="G2" t="s">
+        <v>334</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>274</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{A5E065B3-B151-446B-AFAE-9D4FBBD0510F}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2866,14 +2891,14 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="4" max="4" width="30.42578125" customWidth="1"/>
     <col min="5" max="5" width="58.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2899,7 +2924,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2018</v>
       </c>
@@ -2930,14 +2955,14 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="138.5703125" customWidth="1"/>
     <col min="6" max="6" width="16.42578125" customWidth="1"/>
     <col min="7" max="7" width="40.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2963,7 +2988,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2019</v>
       </c>
@@ -2986,7 +3011,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2019</v>
       </c>
@@ -3009,7 +3034,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>2019</v>
       </c>
@@ -3032,7 +3057,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="409.5">
+    <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>2019</v>
       </c>
@@ -3055,7 +3080,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="409.5">
+    <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>2019</v>
       </c>
@@ -3078,7 +3103,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="409.5">
+    <row r="7" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>2019</v>
       </c>
@@ -3109,7 +3134,7 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="34.140625" customWidth="1"/>
     <col min="3" max="3" width="56.140625" customWidth="1"/>
@@ -3120,7 +3145,7 @@
     <col min="8" max="8" width="67" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75">
+    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -3146,7 +3171,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="12">
         <v>2020</v>
       </c>
@@ -3169,7 +3194,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="12">
         <v>2020</v>
       </c>
@@ -3192,7 +3217,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>2020</v>
       </c>
@@ -3223,13 +3248,13 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="39.7109375" customWidth="1"/>
     <col min="5" max="5" width="118.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -3255,7 +3280,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
         <v>2021</v>
       </c>
@@ -3279,7 +3304,7 @@
       </c>
       <c r="H2" s="7"/>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>2021</v>
       </c>
@@ -3303,7 +3328,7 @@
       </c>
       <c r="H3" s="7"/>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
         <v>2021</v>
       </c>
@@ -3335,7 +3360,7 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.42578125" customWidth="1"/>
     <col min="3" max="4" width="41.5703125" customWidth="1"/>
@@ -3343,7 +3368,7 @@
     <col min="6" max="6" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3369,7 +3394,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.5">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2022</v>
       </c>
@@ -3392,7 +3417,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2022</v>
       </c>
@@ -3415,7 +3440,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>2022</v>
       </c>
@@ -3438,7 +3463,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="409.5">
+    <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>2022</v>
       </c>
@@ -3461,7 +3486,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="409.5">
+    <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>2022</v>
       </c>
@@ -3484,7 +3509,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="409.5">
+    <row r="7" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>2022</v>
       </c>
@@ -3507,7 +3532,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="409.5">
+    <row r="8" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>2022</v>
       </c>
@@ -3538,7 +3563,7 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27.28515625" customWidth="1"/>
     <col min="4" max="4" width="52" customWidth="1"/>
@@ -3546,7 +3571,7 @@
     <col min="6" max="6" width="70.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3572,7 +3597,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2023</v>
       </c>
@@ -3592,7 +3617,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2023</v>
       </c>
@@ -3615,7 +3640,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2023</v>
       </c>
@@ -3632,7 +3657,7 @@
         <v>197</v>
       </c>
       <c r="G4" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
   </sheetData>
@@ -3643,7 +3668,7 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="51.85546875" customWidth="1"/>
     <col min="4" max="4" width="45.5703125" customWidth="1"/>
@@ -3651,7 +3676,7 @@
     <col min="6" max="6" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3677,7 +3702,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -3700,7 +3725,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2024</v>
       </c>
@@ -3720,7 +3745,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2024</v>
       </c>
@@ -3743,7 +3768,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="409.5">
+    <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2024</v>
       </c>
@@ -3763,7 +3788,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="409.5">
+    <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2024</v>
       </c>
@@ -3786,7 +3811,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.75">
+    <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2024</v>
       </c>
@@ -3806,7 +3831,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="409.5">
+    <row r="8" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -3837,7 +3862,7 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.28515625" customWidth="1"/>
     <col min="3" max="3" width="54" customWidth="1"/>
@@ -3847,7 +3872,7 @@
     <col min="8" max="8" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3873,7 +3898,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2025</v>
       </c>
@@ -3893,7 +3918,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="409.5">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -3916,7 +3941,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="409.5">
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2025</v>
       </c>
@@ -3939,7 +3964,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="409.5">
+    <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2025</v>
       </c>
@@ -3962,7 +3987,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="409.5">
+    <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2025</v>
       </c>
@@ -3993,14 +4018,14 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.140625" customWidth="1"/>
     <col min="3" max="3" width="38.140625" customWidth="1"/>
     <col min="5" max="5" width="36.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4026,7 +4051,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -4060,12 +4085,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="48.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4091,7 +4116,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1983</v>
       </c>
@@ -4125,13 +4150,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="10.140625" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4157,7 +4182,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1984</v>
       </c>
@@ -4188,9 +4213,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4216,7 +4241,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1985</v>
       </c>
@@ -4250,12 +4275,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="93.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4281,7 +4306,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1986</v>
       </c>
@@ -4309,9 +4334,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4337,7 +4362,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1988</v>
       </c>
@@ -4365,7 +4390,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.42578125" customWidth="1"/>
     <col min="3" max="3" width="23.7109375" customWidth="1"/>
@@ -4374,7 +4399,7 @@
     <col min="6" max="6" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4400,7 +4425,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="90">
+    <row r="2" spans="1:12" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1989</v>
       </c>
@@ -4418,7 +4443,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="409.5">
+    <row r="3" spans="1:12" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1989</v>
       </c>
@@ -4446,7 +4471,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="30.7109375" customWidth="1"/>
     <col min="4" max="4" width="42" customWidth="1"/>
@@ -4454,7 +4479,7 @@
     <col min="6" max="6" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4480,7 +4505,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.5">
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1992</v>
       </c>
@@ -4500,7 +4525,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="240">
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1992</v>
       </c>
@@ -4514,7 +4539,7 @@
         <v>171</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>11</v>

</xml_diff>